<commit_message>
Correct Table Excel template
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskp_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskp_vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{366F7362-5C97-439B-90C5-A175F6296576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E50B744-D7B2-405A-9DFA-B86A3B4F9360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskp_Beispielbefüllung" sheetId="15" r:id="rId1"/>
@@ -610,7 +610,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -699,85 +699,78 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -867,10 +860,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1196,82 +1185,82 @@
   <sheetData>
     <row r="1" spans="1:42" s="6" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16"/>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="37" t="s">
+      <c r="C1" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="36" t="s">
+      <c r="D1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="36" t="s">
+      <c r="E1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="36" t="s">
+      <c r="H1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="I1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="36" t="s">
+      <c r="J1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="38" t="s">
+      <c r="K1" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="36" t="s">
+      <c r="L1" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="36" t="s">
+      <c r="M1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="36" t="s">
+      <c r="N1" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="38" t="s">
+      <c r="O1" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="39" t="s">
+      <c r="P1" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="36" t="s">
+      <c r="Q1" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="38" t="s">
+      <c r="R1" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="36" t="s">
+      <c r="S1" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="36" t="s">
+      <c r="T1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="U1" s="36" t="s">
+      <c r="U1" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="V1" s="36" t="s">
+      <c r="V1" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="W1" s="40" t="s">
+      <c r="W1" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="X1" s="36" t="s">
+      <c r="X1" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="37" t="s">
+      <c r="Y1" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="37" t="s">
+      <c r="Z1" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="38" t="s">
+      <c r="AA1" s="29" t="s">
         <v>46</v>
       </c>
       <c r="AB1" s="1"/>
@@ -1291,160 +1280,160 @@
       <c r="AP1" s="1"/>
     </row>
     <row r="2" spans="1:42" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="34"/>
-      <c r="B2" s="45" t="s">
+      <c r="A2" s="16"/>
+      <c r="B2" s="40" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="46"/>
-      <c r="D2" s="45" t="s">
+      <c r="C2" s="42"/>
+      <c r="D2" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="45" t="s">
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="40" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="45" t="s">
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="40" t="s">
         <v>22</v>
       </c>
-      <c r="M2" s="47"/>
-      <c r="N2" s="47"/>
-      <c r="O2" s="47"/>
-      <c r="P2" s="47"/>
-      <c r="Q2" s="47"/>
-      <c r="R2" s="46"/>
-      <c r="S2" s="45" t="s">
+      <c r="M2" s="41"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="41"/>
+      <c r="R2" s="42"/>
+      <c r="S2" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="T2" s="47"/>
-      <c r="U2" s="47"/>
-      <c r="V2" s="47"/>
-      <c r="W2" s="47"/>
-      <c r="X2" s="47"/>
-      <c r="Y2" s="47"/>
-      <c r="Z2" s="46"/>
-      <c r="AA2" s="43" t="s">
+      <c r="T2" s="41"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="41"/>
+      <c r="W2" s="41"/>
+      <c r="X2" s="41"/>
+      <c r="Y2" s="41"/>
+      <c r="Z2" s="42"/>
+      <c r="AA2" s="33" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:42" s="1" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35"/>
-      <c r="B3" s="27" t="s">
+      <c r="A3" s="37"/>
+      <c r="B3" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="D3" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="E3" s="28" t="s">
+      <c r="E3" s="35" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="28" t="s">
+      <c r="F3" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="27" t="s">
+      <c r="G3" s="36"/>
+      <c r="H3" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I3" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="J3" s="33" t="s">
+      <c r="J3" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="K3" s="32" t="s">
+      <c r="K3" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="L3" s="27" t="s">
+      <c r="L3" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="M3" s="28" t="s">
+      <c r="M3" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="N3" s="30" t="s">
+      <c r="N3" s="44" t="s">
         <v>54</v>
       </c>
-      <c r="O3" s="30"/>
-      <c r="P3" s="30" t="s">
+      <c r="O3" s="44"/>
+      <c r="P3" s="44" t="s">
         <v>55</v>
       </c>
-      <c r="Q3" s="29" t="s">
+      <c r="Q3" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="R3" s="31" t="s">
+      <c r="R3" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="S3" s="27" t="s">
+      <c r="S3" s="39" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="28" t="s">
+      <c r="T3" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="28" t="s">
+      <c r="U3" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="V3" s="28" t="s">
+      <c r="V3" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="W3" s="28" t="s">
+      <c r="W3" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="X3" s="28" t="s">
+      <c r="X3" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="Y3" s="28" t="s">
+      <c r="Y3" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="Z3" s="32" t="s">
+      <c r="Z3" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="AA3" s="44"/>
+      <c r="AA3" s="34"/>
     </row>
     <row r="4" spans="1:42" s="1" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="35"/>
-      <c r="B4" s="27"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="A4" s="37"/>
+      <c r="B4" s="39"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="35"/>
       <c r="F4" s="7" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="27"/>
-      <c r="I4" s="28"/>
-      <c r="J4" s="33"/>
-      <c r="K4" s="32"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="28"/>
+      <c r="H4" s="39"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="39"/>
+      <c r="M4" s="35"/>
       <c r="N4" s="17" t="s">
         <v>43</v>
       </c>
       <c r="O4" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="29"/>
-      <c r="R4" s="31"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="28"/>
-      <c r="U4" s="28"/>
-      <c r="V4" s="28"/>
-      <c r="W4" s="28"/>
-      <c r="X4" s="28"/>
-      <c r="Y4" s="28"/>
-      <c r="Z4" s="32"/>
-      <c r="AA4" s="44"/>
+      <c r="P4" s="44"/>
+      <c r="Q4" s="43"/>
+      <c r="R4" s="45"/>
+      <c r="S4" s="39"/>
+      <c r="T4" s="35"/>
+      <c r="U4" s="35"/>
+      <c r="V4" s="35"/>
+      <c r="W4" s="35"/>
+      <c r="X4" s="35"/>
+      <c r="Y4" s="35"/>
+      <c r="Z4" s="36"/>
+      <c r="AA4" s="34"/>
     </row>
     <row r="5" spans="1:42" s="8" customFormat="1" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="34"/>
+      <c r="A5" s="16"/>
       <c r="B5" s="18"/>
       <c r="C5" s="19" t="s">
         <v>20</v>
@@ -1477,7 +1466,7 @@
       <c r="O5" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="P5" s="42" t="s">
+      <c r="P5" s="32" t="s">
         <v>19</v>
       </c>
       <c r="Q5" s="21" t="s">
@@ -1544,7 +1533,7 @@
       <c r="X6" s="1"/>
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
-      <c r="AA6" s="41"/>
+      <c r="AA6" s="24"/>
     </row>
     <row r="7" spans="1:42" s="1" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="24"/>
@@ -1562,6 +1551,7 @@
       <c r="S7" s="25"/>
       <c r="T7" s="25"/>
       <c r="V7" s="25"/>
+      <c r="AA7" s="24"/>
     </row>
     <row r="8" spans="1:42" s="1" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
@@ -3719,6 +3709,22 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="M3:M4"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H2:K2"/>
+    <mergeCell ref="L2:R2"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="S2:Z2"/>
+    <mergeCell ref="X3:X4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="V3:V4"/>
+    <mergeCell ref="P3:P4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:U4"/>
     <mergeCell ref="AA3:AA4"/>
     <mergeCell ref="W3:W4"/>
     <mergeCell ref="Z3:Z4"/>
@@ -3733,22 +3739,6 @@
     <mergeCell ref="E3:E4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="X3:X4"/>
-    <mergeCell ref="Q3:Q4"/>
-    <mergeCell ref="V3:V4"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="S3:S4"/>
-    <mergeCell ref="T3:T4"/>
-    <mergeCell ref="U3:U4"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H2:K2"/>
-    <mergeCell ref="L2:R2"/>
-    <mergeCell ref="N3:O3"/>
   </mergeCells>
   <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
@@ -3803,6 +3793,36 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_dlc_DocId xmlns="576ce185-3b2e-4f75-8b7c-efeb82226bea">CS36PAW5EANU-7-19945</_dlc_DocId>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_dlc_DocIdUrl xmlns="576ce185-3b2e-4f75-8b7c-efeb82226bea">
+      <Url>https://vst.tu-dresden.de/planpro/_layouts/15/DocIdRedir.aspx?ID=CS36PAW5EANU-7-19945</Url>
+      <Description>CS36PAW5EANU-7-19945</Description>
+    </_dlc_DocIdUrl>
+    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="6" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="3d4e64bebabe581e87caa1b5e2dea503">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="85eee936267896b8f15e0fd2c7a0c6ca" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -4014,36 +4034,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_dlc_DocId xmlns="576ce185-3b2e-4f75-8b7c-efeb82226bea">CS36PAW5EANU-7-19945</_dlc_DocId>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_dlc_DocIdUrl xmlns="576ce185-3b2e-4f75-8b7c-efeb82226bea">
-      <Url>https://vst.tu-dresden.de/planpro/_layouts/15/DocIdRedir.aspx?ID=CS36PAW5EANU-7-19945</Url>
-      <Description>CS36PAW5EANU-7-19945</Description>
-    </_dlc_DocIdUrl>
-    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9CFCEAE-5A31-4E8D-871E-0FEB90E546B0}">
   <ds:schemaRefs>
@@ -4053,6 +4043,39 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52AA9053-CA78-458B-BFEC-B0A103F9F68C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FBE6F5E-0FD6-4104-B02A-28BCFB30DE46}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF743650-405A-4EB5-9BE5-79180E38FBC9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{044B22B7-1F1B-4A24-A516-CD5663BACD02}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4069,37 +4092,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF743650-405A-4EB5-9BE5-79180E38FBC9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FBE6F5E-0FD6-4104-B02A-28BCFB30DE46}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{52AA9053-CA78-458B-BFEC-B0A103F9F68C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>